<commit_message>
Inclusion of the original price variable
-price_scraping.py, raw_data_OV and data_tratment.py done by Lucía de los Santos
-Update the residual_value_model code to include the original price variable
</commit_message>
<xml_diff>
--- a/vehicle_types.xlsx
+++ b/vehicle_types.xlsx
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="94">
@@ -3727,7 +3727,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>437</v>
+        <v>438</v>
       </c>
     </row>
     <row r="166">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>452</v>
+        <v>453</v>
       </c>
     </row>
     <row r="189">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="204">
@@ -4567,7 +4567,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="208">
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="283">
@@ -10867,7 +10867,7 @@
         </is>
       </c>
       <c r="D522" t="n">
-        <v>468</v>
+        <v>469</v>
       </c>
     </row>
     <row r="523">
@@ -11647,7 +11647,7 @@
         </is>
       </c>
       <c r="D561" t="n">
-        <v>1104</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="562">
@@ -12307,7 +12307,7 @@
         </is>
       </c>
       <c r="D594" t="n">
-        <v>997</v>
+        <v>998</v>
       </c>
     </row>
     <row r="595">
@@ -12347,7 +12347,7 @@
         </is>
       </c>
       <c r="D596" t="n">
-        <v>2754</v>
+        <v>2755</v>
       </c>
     </row>
     <row r="597">
@@ -12647,7 +12647,7 @@
         </is>
       </c>
       <c r="D611" t="n">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="612">
@@ -14407,7 +14407,7 @@
         </is>
       </c>
       <c r="D699" t="n">
-        <v>296</v>
+        <v>297</v>
       </c>
     </row>
     <row r="700">
@@ -14807,7 +14807,7 @@
         </is>
       </c>
       <c r="D719" t="n">
-        <v>726</v>
+        <v>727</v>
       </c>
     </row>
     <row r="720">
@@ -15327,7 +15327,7 @@
         </is>
       </c>
       <c r="D745" t="n">
-        <v>1483</v>
+        <v>1484</v>
       </c>
     </row>
     <row r="746">

</xml_diff>